<commit_message>
update generated data Triggered by 1caf703b23b972b9f73bd5e84d99420bac22b193
</commit_message>
<xml_diff>
--- a/DC-Colos.xlsx
+++ b/DC-Colos.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H343"/>
+  <dimension ref="A1:H342"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11333,12 +11333,12 @@
     <row r="292">
       <c r="A292" s="1" t="inlineStr">
         <is>
-          <t>BUF</t>
+          <t>YYC</t>
         </is>
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>Buffalo, NY, United States</t>
+          <t>Calgary, AB, Canada</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
@@ -11348,35 +11348,35 @@
       </c>
       <c r="D292" t="inlineStr">
         <is>
-          <t>Buffalo</t>
+          <t>Calgary</t>
         </is>
       </c>
       <c r="E292" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F292" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="G292" t="n">
-        <v>42.940498</v>
+        <v>51.113899</v>
       </c>
       <c r="H292" t="n">
-        <v>-78.732201</v>
+        <v>-114.019997</v>
       </c>
     </row>
     <row r="293">
       <c r="A293" s="1" t="inlineStr">
         <is>
-          <t>YYC</t>
+          <t>CLT</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>Calgary, AB, Canada</t>
+          <t>Charlotte, NC, United States</t>
         </is>
       </c>
       <c r="C293" t="inlineStr">
@@ -11386,35 +11386,35 @@
       </c>
       <c r="D293" t="inlineStr">
         <is>
-          <t>Calgary</t>
+          <t>Charlotte</t>
         </is>
       </c>
       <c r="E293" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F293" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G293" t="n">
-        <v>51.113899</v>
+        <v>35.214001</v>
       </c>
       <c r="H293" t="n">
-        <v>-114.019997</v>
+        <v>-80.9431</v>
       </c>
     </row>
     <row r="294">
       <c r="A294" s="1" t="inlineStr">
         <is>
-          <t>CLT</t>
+          <t>ORD</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>Charlotte, NC, United States</t>
+          <t>Chicago, IL, United States</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
@@ -11424,7 +11424,7 @@
       </c>
       <c r="D294" t="inlineStr">
         <is>
-          <t>Charlotte</t>
+          <t>Chicago</t>
         </is>
       </c>
       <c r="E294" t="inlineStr">
@@ -11438,21 +11438,21 @@
         </is>
       </c>
       <c r="G294" t="n">
-        <v>35.214001</v>
+        <v>41.9786</v>
       </c>
       <c r="H294" t="n">
-        <v>-80.9431</v>
+        <v>-87.90479999999999</v>
       </c>
     </row>
     <row r="295">
       <c r="A295" s="1" t="inlineStr">
         <is>
-          <t>ORD</t>
+          <t>CLE</t>
         </is>
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>Chicago, IL, United States</t>
+          <t>Cleveland, OH, United States</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
@@ -11462,7 +11462,7 @@
       </c>
       <c r="D295" t="inlineStr">
         <is>
-          <t>Chicago</t>
+          <t>Cleveland</t>
         </is>
       </c>
       <c r="E295" t="inlineStr">
@@ -11476,21 +11476,21 @@
         </is>
       </c>
       <c r="G295" t="n">
-        <v>41.9786</v>
+        <v>41.411701</v>
       </c>
       <c r="H295" t="n">
-        <v>-87.90479999999999</v>
+        <v>-81.8498</v>
       </c>
     </row>
     <row r="296">
       <c r="A296" s="1" t="inlineStr">
         <is>
-          <t>CLE</t>
+          <t>CMH</t>
         </is>
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>Cleveland, OH, United States</t>
+          <t>Columbus, OH, United States</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
@@ -11500,7 +11500,7 @@
       </c>
       <c r="D296" t="inlineStr">
         <is>
-          <t>Cleveland</t>
+          <t>Columbus</t>
         </is>
       </c>
       <c r="E296" t="inlineStr">
@@ -11514,21 +11514,21 @@
         </is>
       </c>
       <c r="G296" t="n">
-        <v>41.411701</v>
+        <v>39.998001</v>
       </c>
       <c r="H296" t="n">
-        <v>-81.8498</v>
+        <v>-82.891899</v>
       </c>
     </row>
     <row r="297">
       <c r="A297" s="1" t="inlineStr">
         <is>
-          <t>CMH</t>
+          <t>DFW</t>
         </is>
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>Columbus, OH, United States</t>
+          <t>Dallas, TX, United States</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
@@ -11538,7 +11538,7 @@
       </c>
       <c r="D297" t="inlineStr">
         <is>
-          <t>Columbus</t>
+          <t>Dallas-Fort Worth</t>
         </is>
       </c>
       <c r="E297" t="inlineStr">
@@ -11552,21 +11552,21 @@
         </is>
       </c>
       <c r="G297" t="n">
-        <v>39.998001</v>
+        <v>32.896801</v>
       </c>
       <c r="H297" t="n">
-        <v>-82.891899</v>
+        <v>-97.03800200000001</v>
       </c>
     </row>
     <row r="298">
       <c r="A298" s="1" t="inlineStr">
         <is>
-          <t>DFW</t>
+          <t>DEN</t>
         </is>
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>Dallas, TX, United States</t>
+          <t>Denver, CO, United States</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
@@ -11576,7 +11576,7 @@
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t>Dallas-Fort Worth</t>
+          <t>Denver</t>
         </is>
       </c>
       <c r="E298" t="inlineStr">
@@ -11590,21 +11590,21 @@
         </is>
       </c>
       <c r="G298" t="n">
-        <v>32.896801</v>
+        <v>39.861698</v>
       </c>
       <c r="H298" t="n">
-        <v>-97.03800200000001</v>
+        <v>-104.672997</v>
       </c>
     </row>
     <row r="299">
       <c r="A299" s="1" t="inlineStr">
         <is>
-          <t>DEN</t>
+          <t>DTW</t>
         </is>
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>Denver, CO, United States</t>
+          <t>Detroit, MI, United States</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
@@ -11614,7 +11614,7 @@
       </c>
       <c r="D299" t="inlineStr">
         <is>
-          <t>Denver</t>
+          <t>Detroit</t>
         </is>
       </c>
       <c r="E299" t="inlineStr">
@@ -11628,21 +11628,21 @@
         </is>
       </c>
       <c r="G299" t="n">
-        <v>39.861698</v>
+        <v>42.212399</v>
       </c>
       <c r="H299" t="n">
-        <v>-104.672997</v>
+        <v>-83.35340100000001</v>
       </c>
     </row>
     <row r="300">
       <c r="A300" s="1" t="inlineStr">
         <is>
-          <t>DTW</t>
+          <t>RDU</t>
         </is>
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>Detroit, MI, United States</t>
+          <t>Durham, NC, United States</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
@@ -11652,7 +11652,7 @@
       </c>
       <c r="D300" t="inlineStr">
         <is>
-          <t>Detroit</t>
+          <t>Raleigh/Durham</t>
         </is>
       </c>
       <c r="E300" t="inlineStr">
@@ -11666,21 +11666,21 @@
         </is>
       </c>
       <c r="G300" t="n">
-        <v>42.212399</v>
+        <v>35.877602</v>
       </c>
       <c r="H300" t="n">
-        <v>-83.35340100000001</v>
+        <v>-78.787498</v>
       </c>
     </row>
     <row r="301">
       <c r="A301" s="1" t="inlineStr">
         <is>
-          <t>RDU</t>
+          <t>GDL</t>
         </is>
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>Durham, NC, United States</t>
+          <t>Guadalajara, Mexico</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
@@ -11690,35 +11690,35 @@
       </c>
       <c r="D301" t="inlineStr">
         <is>
-          <t>Raleigh/Durham</t>
+          <t>Guadalajara</t>
         </is>
       </c>
       <c r="E301" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F301" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>MX</t>
         </is>
       </c>
       <c r="G301" t="n">
-        <v>35.877602</v>
+        <v>20.521799</v>
       </c>
       <c r="H301" t="n">
-        <v>-78.787498</v>
+        <v>-103.310997</v>
       </c>
     </row>
     <row r="302">
       <c r="A302" s="1" t="inlineStr">
         <is>
-          <t>GDL</t>
+          <t>YHZ</t>
         </is>
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>Guadalajara, Mexico</t>
+          <t>Halifax, Canada</t>
         </is>
       </c>
       <c r="C302" t="inlineStr">
@@ -11728,35 +11728,35 @@
       </c>
       <c r="D302" t="inlineStr">
         <is>
-          <t>Guadalajara</t>
+          <t>Halifax</t>
         </is>
       </c>
       <c r="E302" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F302" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="G302" t="n">
-        <v>20.521799</v>
+        <v>44.880798</v>
       </c>
       <c r="H302" t="n">
-        <v>-103.310997</v>
+        <v>-63.508598</v>
       </c>
     </row>
     <row r="303">
       <c r="A303" s="1" t="inlineStr">
         <is>
-          <t>YHZ</t>
+          <t>HNL</t>
         </is>
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>Halifax, Canada</t>
+          <t>Honolulu, HI, United States</t>
         </is>
       </c>
       <c r="C303" t="inlineStr">
@@ -11766,35 +11766,35 @@
       </c>
       <c r="D303" t="inlineStr">
         <is>
-          <t>Halifax</t>
+          <t>Honolulu</t>
         </is>
       </c>
       <c r="E303" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F303" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G303" t="n">
-        <v>44.880798</v>
+        <v>21.318701</v>
       </c>
       <c r="H303" t="n">
-        <v>-63.508598</v>
+        <v>-157.921997</v>
       </c>
     </row>
     <row r="304">
       <c r="A304" s="1" t="inlineStr">
         <is>
-          <t>HNL</t>
+          <t>IAH</t>
         </is>
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>Honolulu, HI, United States</t>
+          <t>Houston, TX, United States</t>
         </is>
       </c>
       <c r="C304" t="inlineStr">
@@ -11804,7 +11804,7 @@
       </c>
       <c r="D304" t="inlineStr">
         <is>
-          <t>Honolulu</t>
+          <t>Houston</t>
         </is>
       </c>
       <c r="E304" t="inlineStr">
@@ -11818,21 +11818,21 @@
         </is>
       </c>
       <c r="G304" t="n">
-        <v>21.318701</v>
+        <v>29.9844</v>
       </c>
       <c r="H304" t="n">
-        <v>-157.921997</v>
+        <v>-95.34139999999999</v>
       </c>
     </row>
     <row r="305">
       <c r="A305" s="1" t="inlineStr">
         <is>
-          <t>IAH</t>
+          <t>IND</t>
         </is>
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>Houston, TX, United States</t>
+          <t>Indianapolis, IN, United States</t>
         </is>
       </c>
       <c r="C305" t="inlineStr">
@@ -11842,7 +11842,7 @@
       </c>
       <c r="D305" t="inlineStr">
         <is>
-          <t>Houston</t>
+          <t>Indianapolis</t>
         </is>
       </c>
       <c r="E305" t="inlineStr">
@@ -11856,21 +11856,21 @@
         </is>
       </c>
       <c r="G305" t="n">
-        <v>29.9844</v>
+        <v>39.7173</v>
       </c>
       <c r="H305" t="n">
-        <v>-95.34139999999999</v>
+        <v>-86.294403</v>
       </c>
     </row>
     <row r="306">
       <c r="A306" s="1" t="inlineStr">
         <is>
-          <t>IND</t>
+          <t>JAX</t>
         </is>
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>Indianapolis, IN, United States</t>
+          <t>Jacksonville, FL, United States</t>
         </is>
       </c>
       <c r="C306" t="inlineStr">
@@ -11880,7 +11880,7 @@
       </c>
       <c r="D306" t="inlineStr">
         <is>
-          <t>Indianapolis</t>
+          <t>Jacksonville</t>
         </is>
       </c>
       <c r="E306" t="inlineStr">
@@ -11894,21 +11894,21 @@
         </is>
       </c>
       <c r="G306" t="n">
-        <v>39.7173</v>
+        <v>30.494101</v>
       </c>
       <c r="H306" t="n">
-        <v>-86.294403</v>
+        <v>-81.68789700000001</v>
       </c>
     </row>
     <row r="307">
       <c r="A307" s="1" t="inlineStr">
         <is>
-          <t>JAX</t>
+          <t>MCI</t>
         </is>
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>Jacksonville, FL, United States</t>
+          <t>Kansas City, MO, United States</t>
         </is>
       </c>
       <c r="C307" t="inlineStr">
@@ -11918,7 +11918,7 @@
       </c>
       <c r="D307" t="inlineStr">
         <is>
-          <t>Jacksonville</t>
+          <t>Kansas City</t>
         </is>
       </c>
       <c r="E307" t="inlineStr">
@@ -11932,21 +11932,21 @@
         </is>
       </c>
       <c r="G307" t="n">
-        <v>30.494101</v>
+        <v>39.2976</v>
       </c>
       <c r="H307" t="n">
-        <v>-81.68789700000001</v>
+        <v>-94.713898</v>
       </c>
     </row>
     <row r="308">
       <c r="A308" s="1" t="inlineStr">
         <is>
-          <t>MCI</t>
+          <t>KIN</t>
         </is>
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>Kansas City, MO, United States</t>
+          <t>Kingston, Jamaica</t>
         </is>
       </c>
       <c r="C308" t="inlineStr">
@@ -11956,35 +11956,35 @@
       </c>
       <c r="D308" t="inlineStr">
         <is>
-          <t>Kansas City</t>
+          <t>Kingston</t>
         </is>
       </c>
       <c r="E308" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Jamaica</t>
         </is>
       </c>
       <c r="F308" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>JM</t>
         </is>
       </c>
       <c r="G308" t="n">
-        <v>39.2976</v>
+        <v>17.935699</v>
       </c>
       <c r="H308" t="n">
-        <v>-94.713898</v>
+        <v>-76.787498</v>
       </c>
     </row>
     <row r="309">
       <c r="A309" s="1" t="inlineStr">
         <is>
-          <t>KIN</t>
+          <t>LAS</t>
         </is>
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>Kingston, Jamaica</t>
+          <t>Las Vegas, NV, United States</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
@@ -11994,35 +11994,35 @@
       </c>
       <c r="D309" t="inlineStr">
         <is>
-          <t>Kingston</t>
+          <t>Las Vegas</t>
         </is>
       </c>
       <c r="E309" t="inlineStr">
         <is>
-          <t>Jamaica</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F309" t="inlineStr">
         <is>
-          <t>JM</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G309" t="n">
-        <v>17.935699</v>
+        <v>36.080101</v>
       </c>
       <c r="H309" t="n">
-        <v>-76.787498</v>
+        <v>-115.152</v>
       </c>
     </row>
     <row r="310">
       <c r="A310" s="1" t="inlineStr">
         <is>
-          <t>LAS</t>
+          <t>LAX</t>
         </is>
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>Las Vegas, NV, United States</t>
+          <t>Los Angeles, CA, United States</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
@@ -12032,7 +12032,7 @@
       </c>
       <c r="D310" t="inlineStr">
         <is>
-          <t>Las Vegas</t>
+          <t>Los Angeles</t>
         </is>
       </c>
       <c r="E310" t="inlineStr">
@@ -12046,21 +12046,21 @@
         </is>
       </c>
       <c r="G310" t="n">
-        <v>36.080101</v>
+        <v>33.942501</v>
       </c>
       <c r="H310" t="n">
-        <v>-115.152</v>
+        <v>-118.407997</v>
       </c>
     </row>
     <row r="311">
       <c r="A311" s="1" t="inlineStr">
         <is>
-          <t>LAX</t>
+          <t>MEM</t>
         </is>
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>Los Angeles, CA, United States</t>
+          <t>Memphis, TN, United States</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
@@ -12070,7 +12070,7 @@
       </c>
       <c r="D311" t="inlineStr">
         <is>
-          <t>Los Angeles</t>
+          <t>Memphis</t>
         </is>
       </c>
       <c r="E311" t="inlineStr">
@@ -12084,21 +12084,21 @@
         </is>
       </c>
       <c r="G311" t="n">
-        <v>33.942501</v>
+        <v>35.0424</v>
       </c>
       <c r="H311" t="n">
-        <v>-118.407997</v>
+        <v>-89.97669999999999</v>
       </c>
     </row>
     <row r="312">
       <c r="A312" s="1" t="inlineStr">
         <is>
-          <t>MEM</t>
+          <t>MEX</t>
         </is>
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>Memphis, TN, United States</t>
+          <t>Mexico City, Mexico</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
@@ -12108,35 +12108,35 @@
       </c>
       <c r="D312" t="inlineStr">
         <is>
-          <t>Memphis</t>
+          <t>Mexico City</t>
         </is>
       </c>
       <c r="E312" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F312" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>MX</t>
         </is>
       </c>
       <c r="G312" t="n">
-        <v>35.0424</v>
+        <v>19.4363</v>
       </c>
       <c r="H312" t="n">
-        <v>-89.97669999999999</v>
+        <v>-99.072098</v>
       </c>
     </row>
     <row r="313">
       <c r="A313" s="1" t="inlineStr">
         <is>
-          <t>MEX</t>
+          <t>MIA</t>
         </is>
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>Mexico City, Mexico</t>
+          <t>Miami, FL, United States</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
@@ -12146,35 +12146,35 @@
       </c>
       <c r="D313" t="inlineStr">
         <is>
-          <t>Mexico City</t>
+          <t>Miami</t>
         </is>
       </c>
       <c r="E313" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F313" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G313" t="n">
-        <v>19.4363</v>
+        <v>25.7932</v>
       </c>
       <c r="H313" t="n">
-        <v>-99.072098</v>
+        <v>-80.290604</v>
       </c>
     </row>
     <row r="314">
       <c r="A314" s="1" t="inlineStr">
         <is>
-          <t>MIA</t>
+          <t>MSP</t>
         </is>
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>Miami, FL, United States</t>
+          <t>Minneapolis, MN, United States</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
@@ -12184,7 +12184,7 @@
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>Miami</t>
+          <t>Minneapolis</t>
         </is>
       </c>
       <c r="E314" t="inlineStr">
@@ -12198,21 +12198,21 @@
         </is>
       </c>
       <c r="G314" t="n">
-        <v>25.7932</v>
+        <v>44.882</v>
       </c>
       <c r="H314" t="n">
-        <v>-80.290604</v>
+        <v>-93.221802</v>
       </c>
     </row>
     <row r="315">
       <c r="A315" s="1" t="inlineStr">
         <is>
-          <t>MSP</t>
+          <t>YUL</t>
         </is>
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>Minneapolis, MN, United States</t>
+          <t>Montréal, QC, Canada</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
@@ -12222,35 +12222,35 @@
       </c>
       <c r="D315" t="inlineStr">
         <is>
-          <t>Minneapolis</t>
+          <t>Montreal</t>
         </is>
       </c>
       <c r="E315" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F315" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="G315" t="n">
-        <v>44.882</v>
+        <v>45.4706</v>
       </c>
       <c r="H315" t="n">
-        <v>-93.221802</v>
+        <v>-73.740799</v>
       </c>
     </row>
     <row r="316">
       <c r="A316" s="1" t="inlineStr">
         <is>
-          <t>YUL</t>
+          <t>BNA</t>
         </is>
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>Montréal, QC, Canada</t>
+          <t>Nashville, United States</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
@@ -12260,35 +12260,35 @@
       </c>
       <c r="D316" t="inlineStr">
         <is>
-          <t>Montreal</t>
+          <t>Nashville</t>
         </is>
       </c>
       <c r="E316" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F316" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G316" t="n">
-        <v>45.4706</v>
+        <v>36.1245</v>
       </c>
       <c r="H316" t="n">
-        <v>-73.740799</v>
+        <v>-86.6782</v>
       </c>
     </row>
     <row r="317">
       <c r="A317" s="1" t="inlineStr">
         <is>
-          <t>BNA</t>
+          <t>EWR</t>
         </is>
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>Nashville, United States</t>
+          <t>Newark, NJ, United States</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
@@ -12298,7 +12298,7 @@
       </c>
       <c r="D317" t="inlineStr">
         <is>
-          <t>Nashville</t>
+          <t>Newark</t>
         </is>
       </c>
       <c r="E317" t="inlineStr">
@@ -12312,21 +12312,21 @@
         </is>
       </c>
       <c r="G317" t="n">
-        <v>36.1245</v>
+        <v>40.692501</v>
       </c>
       <c r="H317" t="n">
-        <v>-86.6782</v>
+        <v>-74.168701</v>
       </c>
     </row>
     <row r="318">
       <c r="A318" s="1" t="inlineStr">
         <is>
-          <t>EWR</t>
+          <t>ORF</t>
         </is>
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>Newark, NJ, United States</t>
+          <t>Norfolk, VA, United States</t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
@@ -12336,7 +12336,7 @@
       </c>
       <c r="D318" t="inlineStr">
         <is>
-          <t>Newark</t>
+          <t>Norfolk</t>
         </is>
       </c>
       <c r="E318" t="inlineStr">
@@ -12350,21 +12350,21 @@
         </is>
       </c>
       <c r="G318" t="n">
-        <v>40.692501</v>
+        <v>36.8946</v>
       </c>
       <c r="H318" t="n">
-        <v>-74.168701</v>
+        <v>-76.20120199999999</v>
       </c>
     </row>
     <row r="319">
       <c r="A319" s="1" t="inlineStr">
         <is>
-          <t>ORF</t>
+          <t>OKC</t>
         </is>
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>Norfolk, VA, United States</t>
+          <t>Oklahoma City, OK, United States</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
@@ -12374,7 +12374,7 @@
       </c>
       <c r="D319" t="inlineStr">
         <is>
-          <t>Norfolk</t>
+          <t>Oklahoma City</t>
         </is>
       </c>
       <c r="E319" t="inlineStr">
@@ -12388,21 +12388,21 @@
         </is>
       </c>
       <c r="G319" t="n">
-        <v>36.8946</v>
+        <v>35.393101</v>
       </c>
       <c r="H319" t="n">
-        <v>-76.20120199999999</v>
+        <v>-97.6007</v>
       </c>
     </row>
     <row r="320">
       <c r="A320" s="1" t="inlineStr">
         <is>
-          <t>OKC</t>
+          <t>OMA</t>
         </is>
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>Oklahoma City, OK, United States</t>
+          <t>Omaha, NE, United States</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
@@ -12412,7 +12412,7 @@
       </c>
       <c r="D320" t="inlineStr">
         <is>
-          <t>Oklahoma City</t>
+          <t>Omaha</t>
         </is>
       </c>
       <c r="E320" t="inlineStr">
@@ -12426,21 +12426,21 @@
         </is>
       </c>
       <c r="G320" t="n">
-        <v>35.393101</v>
+        <v>41.3032</v>
       </c>
       <c r="H320" t="n">
-        <v>-97.6007</v>
+        <v>-95.894096</v>
       </c>
     </row>
     <row r="321">
       <c r="A321" s="1" t="inlineStr">
         <is>
-          <t>OMA</t>
+          <t>PHL</t>
         </is>
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>Omaha, NE, United States</t>
+          <t>Philadelphia, United States</t>
         </is>
       </c>
       <c r="C321" t="inlineStr">
@@ -12450,7 +12450,7 @@
       </c>
       <c r="D321" t="inlineStr">
         <is>
-          <t>Omaha</t>
+          <t>Philadelphia</t>
         </is>
       </c>
       <c r="E321" t="inlineStr">
@@ -12464,21 +12464,21 @@
         </is>
       </c>
       <c r="G321" t="n">
-        <v>41.3032</v>
+        <v>39.871899</v>
       </c>
       <c r="H321" t="n">
-        <v>-95.894096</v>
+        <v>-75.241096</v>
       </c>
     </row>
     <row r="322">
       <c r="A322" s="1" t="inlineStr">
         <is>
-          <t>PHL</t>
+          <t>PHX</t>
         </is>
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>Philadelphia, United States</t>
+          <t>Phoenix, AZ, United States</t>
         </is>
       </c>
       <c r="C322" t="inlineStr">
@@ -12488,7 +12488,7 @@
       </c>
       <c r="D322" t="inlineStr">
         <is>
-          <t>Philadelphia</t>
+          <t>Phoenix</t>
         </is>
       </c>
       <c r="E322" t="inlineStr">
@@ -12502,21 +12502,21 @@
         </is>
       </c>
       <c r="G322" t="n">
-        <v>39.871899</v>
+        <v>33.434299</v>
       </c>
       <c r="H322" t="n">
-        <v>-75.241096</v>
+        <v>-112.012001</v>
       </c>
     </row>
     <row r="323">
       <c r="A323" s="1" t="inlineStr">
         <is>
-          <t>PHX</t>
+          <t>PIT</t>
         </is>
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>Phoenix, AZ, United States</t>
+          <t>Pittsburgh, PA, United States</t>
         </is>
       </c>
       <c r="C323" t="inlineStr">
@@ -12526,7 +12526,7 @@
       </c>
       <c r="D323" t="inlineStr">
         <is>
-          <t>Phoenix</t>
+          <t>Pittsburgh</t>
         </is>
       </c>
       <c r="E323" t="inlineStr">
@@ -12540,21 +12540,21 @@
         </is>
       </c>
       <c r="G323" t="n">
-        <v>33.434299</v>
+        <v>40.491501</v>
       </c>
       <c r="H323" t="n">
-        <v>-112.012001</v>
+        <v>-80.23290299999999</v>
       </c>
     </row>
     <row r="324">
       <c r="A324" s="1" t="inlineStr">
         <is>
-          <t>PIT</t>
+          <t>PDX</t>
         </is>
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>Pittsburgh, PA, United States</t>
+          <t>Portland, OR, United States</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
@@ -12564,7 +12564,7 @@
       </c>
       <c r="D324" t="inlineStr">
         <is>
-          <t>Pittsburgh</t>
+          <t>Portland</t>
         </is>
       </c>
       <c r="E324" t="inlineStr">
@@ -12578,21 +12578,21 @@
         </is>
       </c>
       <c r="G324" t="n">
-        <v>40.491501</v>
+        <v>45.588699</v>
       </c>
       <c r="H324" t="n">
-        <v>-80.23290299999999</v>
+        <v>-122.598</v>
       </c>
     </row>
     <row r="325">
       <c r="A325" s="1" t="inlineStr">
         <is>
-          <t>PDX</t>
+          <t>QRO</t>
         </is>
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>Portland, OR, United States</t>
+          <t>Queretaro, MX, Mexico</t>
         </is>
       </c>
       <c r="C325" t="inlineStr">
@@ -12602,35 +12602,35 @@
       </c>
       <c r="D325" t="inlineStr">
         <is>
-          <t>Portland</t>
+          <t>Queretaro</t>
         </is>
       </c>
       <c r="E325" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F325" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>MX</t>
         </is>
       </c>
       <c r="G325" t="n">
-        <v>45.588699</v>
+        <v>20.6173</v>
       </c>
       <c r="H325" t="n">
-        <v>-122.598</v>
+        <v>-100.185997</v>
       </c>
     </row>
     <row r="326">
       <c r="A326" s="1" t="inlineStr">
         <is>
-          <t>QRO</t>
+          <t>RIC</t>
         </is>
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>Queretaro, MX, Mexico</t>
+          <t>Richmond, VA, United States</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
@@ -12640,35 +12640,35 @@
       </c>
       <c r="D326" t="inlineStr">
         <is>
-          <t>Queretaro</t>
+          <t>Richmond</t>
         </is>
       </c>
       <c r="E326" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F326" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G326" t="n">
-        <v>20.6173</v>
+        <v>37.505199</v>
       </c>
       <c r="H326" t="n">
-        <v>-100.185997</v>
+        <v>-77.31970200000001</v>
       </c>
     </row>
     <row r="327">
       <c r="A327" s="1" t="inlineStr">
         <is>
-          <t>RIC</t>
+          <t>SMF</t>
         </is>
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>Richmond, VA, United States</t>
+          <t>Sacramento, CA, United States</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
@@ -12678,7 +12678,7 @@
       </c>
       <c r="D327" t="inlineStr">
         <is>
-          <t>Richmond</t>
+          <t>Sacramento</t>
         </is>
       </c>
       <c r="E327" t="inlineStr">
@@ -12692,21 +12692,21 @@
         </is>
       </c>
       <c r="G327" t="n">
-        <v>37.505199</v>
+        <v>38.6954</v>
       </c>
       <c r="H327" t="n">
-        <v>-77.31970200000001</v>
+        <v>-121.591003</v>
       </c>
     </row>
     <row r="328">
       <c r="A328" s="1" t="inlineStr">
         <is>
-          <t>SMF</t>
+          <t>SLC</t>
         </is>
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>Sacramento, CA, United States</t>
+          <t>Salt Lake City, UT, United States</t>
         </is>
       </c>
       <c r="C328" t="inlineStr">
@@ -12716,7 +12716,7 @@
       </c>
       <c r="D328" t="inlineStr">
         <is>
-          <t>Sacramento</t>
+          <t>Salt Lake City</t>
         </is>
       </c>
       <c r="E328" t="inlineStr">
@@ -12730,21 +12730,21 @@
         </is>
       </c>
       <c r="G328" t="n">
-        <v>38.6954</v>
+        <v>40.788399</v>
       </c>
       <c r="H328" t="n">
-        <v>-121.591003</v>
+        <v>-111.977997</v>
       </c>
     </row>
     <row r="329">
       <c r="A329" s="1" t="inlineStr">
         <is>
-          <t>SLC</t>
+          <t>SAT</t>
         </is>
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>Salt Lake City, UT, United States</t>
+          <t>San Antonio, TX, United States</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
@@ -12754,7 +12754,7 @@
       </c>
       <c r="D329" t="inlineStr">
         <is>
-          <t>Salt Lake City</t>
+          <t>San Antonio</t>
         </is>
       </c>
       <c r="E329" t="inlineStr">
@@ -12768,21 +12768,21 @@
         </is>
       </c>
       <c r="G329" t="n">
-        <v>40.788399</v>
+        <v>29.533701</v>
       </c>
       <c r="H329" t="n">
-        <v>-111.977997</v>
+        <v>-98.469803</v>
       </c>
     </row>
     <row r="330">
       <c r="A330" s="1" t="inlineStr">
         <is>
-          <t>SAT</t>
+          <t>SAN</t>
         </is>
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>San Antonio, TX, United States</t>
+          <t>San Diego, CA, United States</t>
         </is>
       </c>
       <c r="C330" t="inlineStr">
@@ -12792,7 +12792,7 @@
       </c>
       <c r="D330" t="inlineStr">
         <is>
-          <t>San Antonio</t>
+          <t>San Diego</t>
         </is>
       </c>
       <c r="E330" t="inlineStr">
@@ -12806,21 +12806,21 @@
         </is>
       </c>
       <c r="G330" t="n">
-        <v>29.533701</v>
+        <v>32.733601</v>
       </c>
       <c r="H330" t="n">
-        <v>-98.469803</v>
+        <v>-117.190002</v>
       </c>
     </row>
     <row r="331">
       <c r="A331" s="1" t="inlineStr">
         <is>
-          <t>SAN</t>
+          <t>SFO</t>
         </is>
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>San Diego, CA, United States</t>
+          <t>San Francisco, CA, United States</t>
         </is>
       </c>
       <c r="C331" t="inlineStr">
@@ -12830,7 +12830,7 @@
       </c>
       <c r="D331" t="inlineStr">
         <is>
-          <t>San Diego</t>
+          <t>San Francisco</t>
         </is>
       </c>
       <c r="E331" t="inlineStr">
@@ -12844,21 +12844,21 @@
         </is>
       </c>
       <c r="G331" t="n">
-        <v>32.733601</v>
+        <v>37.618999</v>
       </c>
       <c r="H331" t="n">
-        <v>-117.190002</v>
+        <v>-122.375</v>
       </c>
     </row>
     <row r="332">
       <c r="A332" s="1" t="inlineStr">
         <is>
-          <t>SFO</t>
+          <t>SJC</t>
         </is>
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>San Francisco, CA, United States</t>
+          <t>San Jose, CA, United States</t>
         </is>
       </c>
       <c r="C332" t="inlineStr">
@@ -12868,7 +12868,7 @@
       </c>
       <c r="D332" t="inlineStr">
         <is>
-          <t>San Francisco</t>
+          <t>San Jose</t>
         </is>
       </c>
       <c r="E332" t="inlineStr">
@@ -12882,21 +12882,21 @@
         </is>
       </c>
       <c r="G332" t="n">
-        <v>37.618999</v>
+        <v>37.362598</v>
       </c>
       <c r="H332" t="n">
-        <v>-122.375</v>
+        <v>-121.929001</v>
       </c>
     </row>
     <row r="333">
       <c r="A333" s="1" t="inlineStr">
         <is>
-          <t>SJC</t>
+          <t>YXE</t>
         </is>
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>San Jose, CA, United States</t>
+          <t>Saskatoon, SK, Canada</t>
         </is>
       </c>
       <c r="C333" t="inlineStr">
@@ -12906,35 +12906,35 @@
       </c>
       <c r="D333" t="inlineStr">
         <is>
-          <t>San Jose</t>
+          <t>Saskatoon</t>
         </is>
       </c>
       <c r="E333" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F333" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="G333" t="n">
-        <v>37.362598</v>
+        <v>52.170799</v>
       </c>
       <c r="H333" t="n">
-        <v>-121.929001</v>
+        <v>-106.699997</v>
       </c>
     </row>
     <row r="334">
       <c r="A334" s="1" t="inlineStr">
         <is>
-          <t>YXE</t>
+          <t>SEA</t>
         </is>
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>Saskatoon, SK, Canada</t>
+          <t>Seattle, WA, United States</t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
@@ -12944,35 +12944,35 @@
       </c>
       <c r="D334" t="inlineStr">
         <is>
-          <t>Saskatoon</t>
+          <t>Seattle</t>
         </is>
       </c>
       <c r="E334" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F334" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G334" t="n">
-        <v>52.170799</v>
+        <v>47.449001</v>
       </c>
       <c r="H334" t="n">
-        <v>-106.699997</v>
+        <v>-122.308998</v>
       </c>
     </row>
     <row r="335">
       <c r="A335" s="1" t="inlineStr">
         <is>
-          <t>SEA</t>
+          <t>FSD</t>
         </is>
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>Seattle, WA, United States</t>
+          <t>Sioux Falls, SD, United States</t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
@@ -12982,7 +12982,7 @@
       </c>
       <c r="D335" t="inlineStr">
         <is>
-          <t>Seattle</t>
+          <t>Sioux Falls</t>
         </is>
       </c>
       <c r="E335" t="inlineStr">
@@ -12996,21 +12996,21 @@
         </is>
       </c>
       <c r="G335" t="n">
-        <v>47.449001</v>
+        <v>43.582001</v>
       </c>
       <c r="H335" t="n">
-        <v>-122.308998</v>
+        <v>-96.74189800000001</v>
       </c>
     </row>
     <row r="336">
       <c r="A336" s="1" t="inlineStr">
         <is>
-          <t>FSD</t>
+          <t>STL</t>
         </is>
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>Sioux Falls, SD, United States</t>
+          <t>St. Louis, MO, United States</t>
         </is>
       </c>
       <c r="C336" t="inlineStr">
@@ -13020,7 +13020,7 @@
       </c>
       <c r="D336" t="inlineStr">
         <is>
-          <t>Sioux Falls</t>
+          <t>St Louis</t>
         </is>
       </c>
       <c r="E336" t="inlineStr">
@@ -13034,21 +13034,21 @@
         </is>
       </c>
       <c r="G336" t="n">
-        <v>43.582001</v>
+        <v>38.748699</v>
       </c>
       <c r="H336" t="n">
-        <v>-96.74189800000001</v>
+        <v>-90.370003</v>
       </c>
     </row>
     <row r="337">
       <c r="A337" s="1" t="inlineStr">
         <is>
-          <t>STL</t>
+          <t>TLH</t>
         </is>
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>St. Louis, MO, United States</t>
+          <t>Tallahassee, FL, United States</t>
         </is>
       </c>
       <c r="C337" t="inlineStr">
@@ -13058,7 +13058,7 @@
       </c>
       <c r="D337" t="inlineStr">
         <is>
-          <t>St Louis</t>
+          <t>Tallahassee</t>
         </is>
       </c>
       <c r="E337" t="inlineStr">
@@ -13072,21 +13072,21 @@
         </is>
       </c>
       <c r="G337" t="n">
-        <v>38.748699</v>
+        <v>30.3965</v>
       </c>
       <c r="H337" t="n">
-        <v>-90.370003</v>
+        <v>-84.35030399999999</v>
       </c>
     </row>
     <row r="338">
       <c r="A338" s="1" t="inlineStr">
         <is>
-          <t>TLH</t>
+          <t>TPA</t>
         </is>
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t>Tallahassee, FL, United States</t>
+          <t>Tampa, FL, United States</t>
         </is>
       </c>
       <c r="C338" t="inlineStr">
@@ -13096,7 +13096,7 @@
       </c>
       <c r="D338" t="inlineStr">
         <is>
-          <t>Tallahassee</t>
+          <t>Tampa</t>
         </is>
       </c>
       <c r="E338" t="inlineStr">
@@ -13110,21 +13110,21 @@
         </is>
       </c>
       <c r="G338" t="n">
-        <v>30.3965</v>
+        <v>27.9755</v>
       </c>
       <c r="H338" t="n">
-        <v>-84.35030399999999</v>
+        <v>-82.533203</v>
       </c>
     </row>
     <row r="339">
       <c r="A339" s="1" t="inlineStr">
         <is>
-          <t>TPA</t>
+          <t>YYZ</t>
         </is>
       </c>
       <c r="B339" t="inlineStr">
         <is>
-          <t>Tampa, FL, United States</t>
+          <t>Toronto, ON, Canada</t>
         </is>
       </c>
       <c r="C339" t="inlineStr">
@@ -13134,35 +13134,35 @@
       </c>
       <c r="D339" t="inlineStr">
         <is>
-          <t>Tampa</t>
+          <t>Toronto</t>
         </is>
       </c>
       <c r="E339" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F339" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="G339" t="n">
-        <v>27.9755</v>
+        <v>43.6772</v>
       </c>
       <c r="H339" t="n">
-        <v>-82.533203</v>
+        <v>-79.6306</v>
       </c>
     </row>
     <row r="340">
       <c r="A340" s="1" t="inlineStr">
         <is>
-          <t>YYZ</t>
+          <t>YVR</t>
         </is>
       </c>
       <c r="B340" t="inlineStr">
         <is>
-          <t>Toronto, ON, Canada</t>
+          <t>Vancouver, BC, Canada</t>
         </is>
       </c>
       <c r="C340" t="inlineStr">
@@ -13172,7 +13172,7 @@
       </c>
       <c r="D340" t="inlineStr">
         <is>
-          <t>Toronto</t>
+          <t>Vancouver</t>
         </is>
       </c>
       <c r="E340" t="inlineStr">
@@ -13186,21 +13186,21 @@
         </is>
       </c>
       <c r="G340" t="n">
-        <v>43.6772</v>
+        <v>49.193901</v>
       </c>
       <c r="H340" t="n">
-        <v>-79.6306</v>
+        <v>-123.183998</v>
       </c>
     </row>
     <row r="341">
       <c r="A341" s="1" t="inlineStr">
         <is>
-          <t>YVR</t>
+          <t>YWG</t>
         </is>
       </c>
       <c r="B341" t="inlineStr">
         <is>
-          <t>Vancouver, BC, Canada</t>
+          <t>Winnipeg, MB, Canada</t>
         </is>
       </c>
       <c r="C341" t="inlineStr">
@@ -13210,7 +13210,7 @@
       </c>
       <c r="D341" t="inlineStr">
         <is>
-          <t>Vancouver</t>
+          <t>Winnipeg</t>
         </is>
       </c>
       <c r="E341" t="inlineStr">
@@ -13224,21 +13224,21 @@
         </is>
       </c>
       <c r="G341" t="n">
-        <v>49.193901</v>
+        <v>49.91</v>
       </c>
       <c r="H341" t="n">
-        <v>-123.183998</v>
+        <v>-97.23989899999999</v>
       </c>
     </row>
     <row r="342">
       <c r="A342" s="1" t="inlineStr">
         <is>
-          <t>YWG</t>
+          <t>CVG</t>
         </is>
       </c>
       <c r="B342" t="inlineStr">
         <is>
-          <t>Winnipeg, MB, Canada</t>
+          <t>Cincinnati, United States</t>
         </is>
       </c>
       <c r="C342" t="inlineStr">
@@ -13248,61 +13248,23 @@
       </c>
       <c r="D342" t="inlineStr">
         <is>
-          <t>Winnipeg</t>
+          <t>Hebron</t>
         </is>
       </c>
       <c r="E342" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F342" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G342" t="n">
-        <v>49.91</v>
+        <v>39.048801</v>
       </c>
       <c r="H342" t="n">
-        <v>-97.23989899999999</v>
-      </c>
-    </row>
-    <row r="343">
-      <c r="A343" s="1" t="inlineStr">
-        <is>
-          <t>CVG</t>
-        </is>
-      </c>
-      <c r="B343" t="inlineStr">
-        <is>
-          <t>Cincinnati, United States</t>
-        </is>
-      </c>
-      <c r="C343" t="inlineStr">
-        <is>
-          <t>North America</t>
-        </is>
-      </c>
-      <c r="D343" t="inlineStr">
-        <is>
-          <t>Hebron</t>
-        </is>
-      </c>
-      <c r="E343" t="inlineStr">
-        <is>
-          <t>United States</t>
-        </is>
-      </c>
-      <c r="F343" t="inlineStr">
-        <is>
-          <t>US</t>
-        </is>
-      </c>
-      <c r="G343" t="n">
-        <v>39.048801</v>
-      </c>
-      <c r="H343" t="n">
         <v>-84.667801</v>
       </c>
     </row>

</xml_diff>

<commit_message>
update generated data Triggered by 8227d4485ba1e0e3b1a392a26a51582a42b4f123
</commit_message>
<xml_diff>
--- a/DC-Colos.xlsx
+++ b/DC-Colos.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H342"/>
+  <dimension ref="A1:H343"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10869,50 +10869,50 @@
     <row r="280">
       <c r="A280" s="1" t="inlineStr">
         <is>
-          <t>ABQ</t>
+          <t>JAI</t>
         </is>
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>Albuquerque, United States</t>
+          <t>“Jaipur”, India</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>North America</t>
+          <t>Asia Pacific</t>
         </is>
       </c>
       <c r="D280" t="inlineStr">
         <is>
-          <t>Albuquerque</t>
+          <t>Jaipur</t>
         </is>
       </c>
       <c r="E280" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F280" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>IN</t>
         </is>
       </c>
       <c r="G280" t="n">
-        <v>35.040199</v>
+        <v>26.8242</v>
       </c>
       <c r="H280" t="n">
-        <v>-106.609001</v>
+        <v>75.812202</v>
       </c>
     </row>
     <row r="281">
       <c r="A281" s="1" t="inlineStr">
         <is>
-          <t>ANC</t>
+          <t>ABQ</t>
         </is>
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>Anchorage, United States</t>
+          <t>Albuquerque, United States</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
@@ -10922,7 +10922,7 @@
       </c>
       <c r="D281" t="inlineStr">
         <is>
-          <t>Anchorage</t>
+          <t>Albuquerque</t>
         </is>
       </c>
       <c r="E281" t="inlineStr">
@@ -10936,21 +10936,21 @@
         </is>
       </c>
       <c r="G281" t="n">
-        <v>61.1744</v>
+        <v>35.040199</v>
       </c>
       <c r="H281" t="n">
-        <v>-149.996002</v>
+        <v>-106.609001</v>
       </c>
     </row>
     <row r="282">
       <c r="A282" s="1" t="inlineStr">
         <is>
-          <t>IAD</t>
+          <t>ANC</t>
         </is>
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>Ashburn, United States</t>
+          <t>Anchorage, United States</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
@@ -10960,7 +10960,7 @@
       </c>
       <c r="D282" t="inlineStr">
         <is>
-          <t>Dulles</t>
+          <t>Anchorage</t>
         </is>
       </c>
       <c r="E282" t="inlineStr">
@@ -10974,21 +10974,21 @@
         </is>
       </c>
       <c r="G282" t="n">
-        <v>38.9445</v>
+        <v>61.1744</v>
       </c>
       <c r="H282" t="n">
-        <v>-77.455803</v>
+        <v>-149.996002</v>
       </c>
     </row>
     <row r="283">
       <c r="A283" s="1" t="inlineStr">
         <is>
-          <t>ATL</t>
+          <t>IAD</t>
         </is>
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>Atlanta, United States</t>
+          <t>Ashburn, United States</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
@@ -10998,7 +10998,7 @@
       </c>
       <c r="D283" t="inlineStr">
         <is>
-          <t>Atlanta</t>
+          <t>Dulles</t>
         </is>
       </c>
       <c r="E283" t="inlineStr">
@@ -11012,21 +11012,21 @@
         </is>
       </c>
       <c r="G283" t="n">
-        <v>33.6367</v>
+        <v>38.9445</v>
       </c>
       <c r="H283" t="n">
-        <v>-84.428101</v>
+        <v>-77.455803</v>
       </c>
     </row>
     <row r="284">
       <c r="A284" s="1" t="inlineStr">
         <is>
-          <t>AUS</t>
+          <t>ATL</t>
         </is>
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>Austin, United States</t>
+          <t>Atlanta, United States</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
@@ -11036,7 +11036,7 @@
       </c>
       <c r="D284" t="inlineStr">
         <is>
-          <t>Austin</t>
+          <t>Atlanta</t>
         </is>
       </c>
       <c r="E284" t="inlineStr">
@@ -11050,21 +11050,21 @@
         </is>
       </c>
       <c r="G284" t="n">
-        <v>30.1945</v>
+        <v>33.6367</v>
       </c>
       <c r="H284" t="n">
-        <v>-97.669899</v>
+        <v>-84.428101</v>
       </c>
     </row>
     <row r="285">
       <c r="A285" s="1" t="inlineStr">
         <is>
-          <t>BGR</t>
+          <t>AUS</t>
         </is>
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>Bangor, United States</t>
+          <t>Austin, United States</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
@@ -11074,7 +11074,7 @@
       </c>
       <c r="D285" t="inlineStr">
         <is>
-          <t>Bangor</t>
+          <t>Austin</t>
         </is>
       </c>
       <c r="E285" t="inlineStr">
@@ -11088,21 +11088,21 @@
         </is>
       </c>
       <c r="G285" t="n">
-        <v>44.8074</v>
+        <v>30.1945</v>
       </c>
       <c r="H285" t="n">
-        <v>-68.828102</v>
+        <v>-97.669899</v>
       </c>
     </row>
     <row r="286">
       <c r="A286" s="1" t="inlineStr">
         <is>
-          <t>BOS</t>
+          <t>BGR</t>
         </is>
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>Boston, United States</t>
+          <t>Bangor, United States</t>
         </is>
       </c>
       <c r="C286" t="inlineStr">
@@ -11112,7 +11112,7 @@
       </c>
       <c r="D286" t="inlineStr">
         <is>
-          <t>Boston</t>
+          <t>Bangor</t>
         </is>
       </c>
       <c r="E286" t="inlineStr">
@@ -11126,21 +11126,21 @@
         </is>
       </c>
       <c r="G286" t="n">
-        <v>42.3643</v>
+        <v>44.8074</v>
       </c>
       <c r="H286" t="n">
-        <v>-71.00520299999999</v>
+        <v>-68.828102</v>
       </c>
     </row>
     <row r="287">
       <c r="A287" s="1" t="inlineStr">
         <is>
-          <t>YYC</t>
+          <t>BOS</t>
         </is>
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>Calgary, Canada</t>
+          <t>Boston, United States</t>
         </is>
       </c>
       <c r="C287" t="inlineStr">
@@ -11150,35 +11150,35 @@
       </c>
       <c r="D287" t="inlineStr">
         <is>
-          <t>Calgary</t>
+          <t>Boston</t>
         </is>
       </c>
       <c r="E287" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F287" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G287" t="n">
-        <v>51.113899</v>
+        <v>42.3643</v>
       </c>
       <c r="H287" t="n">
-        <v>-114.019997</v>
+        <v>-71.00520299999999</v>
       </c>
     </row>
     <row r="288">
       <c r="A288" s="1" t="inlineStr">
         <is>
-          <t>CLT</t>
+          <t>YYC</t>
         </is>
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>Charlotte, United States</t>
+          <t>Calgary, Canada</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
@@ -11188,35 +11188,35 @@
       </c>
       <c r="D288" t="inlineStr">
         <is>
-          <t>Charlotte</t>
+          <t>Calgary</t>
         </is>
       </c>
       <c r="E288" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F288" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="G288" t="n">
-        <v>35.214001</v>
+        <v>51.113899</v>
       </c>
       <c r="H288" t="n">
-        <v>-80.9431</v>
+        <v>-114.019997</v>
       </c>
     </row>
     <row r="289">
       <c r="A289" s="1" t="inlineStr">
         <is>
-          <t>ORD</t>
+          <t>CLT</t>
         </is>
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>Chicago, United States</t>
+          <t>Charlotte, United States</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
@@ -11226,7 +11226,7 @@
       </c>
       <c r="D289" t="inlineStr">
         <is>
-          <t>Chicago</t>
+          <t>Charlotte</t>
         </is>
       </c>
       <c r="E289" t="inlineStr">
@@ -11240,21 +11240,21 @@
         </is>
       </c>
       <c r="G289" t="n">
-        <v>41.9786</v>
+        <v>35.214001</v>
       </c>
       <c r="H289" t="n">
-        <v>-87.90479999999999</v>
+        <v>-80.9431</v>
       </c>
     </row>
     <row r="290">
       <c r="A290" s="1" t="inlineStr">
         <is>
-          <t>CLE</t>
+          <t>ORD</t>
         </is>
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>Cleveland, United States</t>
+          <t>Chicago, United States</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
@@ -11264,7 +11264,7 @@
       </c>
       <c r="D290" t="inlineStr">
         <is>
-          <t>Cleveland</t>
+          <t>Chicago</t>
         </is>
       </c>
       <c r="E290" t="inlineStr">
@@ -11278,21 +11278,21 @@
         </is>
       </c>
       <c r="G290" t="n">
-        <v>41.411701</v>
+        <v>41.9786</v>
       </c>
       <c r="H290" t="n">
-        <v>-81.8498</v>
+        <v>-87.90479999999999</v>
       </c>
     </row>
     <row r="291">
       <c r="A291" s="1" t="inlineStr">
         <is>
-          <t>CMH</t>
+          <t>CLE</t>
         </is>
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>Columbus, United States</t>
+          <t>Cleveland, United States</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
@@ -11302,7 +11302,7 @@
       </c>
       <c r="D291" t="inlineStr">
         <is>
-          <t>Columbus</t>
+          <t>Cleveland</t>
         </is>
       </c>
       <c r="E291" t="inlineStr">
@@ -11316,21 +11316,21 @@
         </is>
       </c>
       <c r="G291" t="n">
-        <v>39.998001</v>
+        <v>41.411701</v>
       </c>
       <c r="H291" t="n">
-        <v>-82.891899</v>
+        <v>-81.8498</v>
       </c>
     </row>
     <row r="292">
       <c r="A292" s="1" t="inlineStr">
         <is>
-          <t>DFW</t>
+          <t>CMH</t>
         </is>
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>Dallas, United States</t>
+          <t>Columbus, United States</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
@@ -11340,7 +11340,7 @@
       </c>
       <c r="D292" t="inlineStr">
         <is>
-          <t>Dallas-Fort Worth</t>
+          <t>Columbus</t>
         </is>
       </c>
       <c r="E292" t="inlineStr">
@@ -11354,21 +11354,21 @@
         </is>
       </c>
       <c r="G292" t="n">
-        <v>32.896801</v>
+        <v>39.998001</v>
       </c>
       <c r="H292" t="n">
-        <v>-97.03800200000001</v>
+        <v>-82.891899</v>
       </c>
     </row>
     <row r="293">
       <c r="A293" s="1" t="inlineStr">
         <is>
-          <t>DEN</t>
+          <t>DFW</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>Denver, United States</t>
+          <t>Dallas, United States</t>
         </is>
       </c>
       <c r="C293" t="inlineStr">
@@ -11378,7 +11378,7 @@
       </c>
       <c r="D293" t="inlineStr">
         <is>
-          <t>Denver</t>
+          <t>Dallas-Fort Worth</t>
         </is>
       </c>
       <c r="E293" t="inlineStr">
@@ -11392,21 +11392,21 @@
         </is>
       </c>
       <c r="G293" t="n">
-        <v>39.861698</v>
+        <v>32.896801</v>
       </c>
       <c r="H293" t="n">
-        <v>-104.672997</v>
+        <v>-97.03800200000001</v>
       </c>
     </row>
     <row r="294">
       <c r="A294" s="1" t="inlineStr">
         <is>
-          <t>DTW</t>
+          <t>DEN</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>Detroit, United States</t>
+          <t>Denver, United States</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
@@ -11416,7 +11416,7 @@
       </c>
       <c r="D294" t="inlineStr">
         <is>
-          <t>Detroit</t>
+          <t>Denver</t>
         </is>
       </c>
       <c r="E294" t="inlineStr">
@@ -11430,21 +11430,21 @@
         </is>
       </c>
       <c r="G294" t="n">
-        <v>42.212399</v>
+        <v>39.861698</v>
       </c>
       <c r="H294" t="n">
-        <v>-83.35340100000001</v>
+        <v>-104.672997</v>
       </c>
     </row>
     <row r="295">
       <c r="A295" s="1" t="inlineStr">
         <is>
-          <t>RDU</t>
+          <t>DTW</t>
         </is>
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>Durham, United States</t>
+          <t>Detroit, United States</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
@@ -11454,7 +11454,7 @@
       </c>
       <c r="D295" t="inlineStr">
         <is>
-          <t>Raleigh/Durham</t>
+          <t>Detroit</t>
         </is>
       </c>
       <c r="E295" t="inlineStr">
@@ -11468,21 +11468,21 @@
         </is>
       </c>
       <c r="G295" t="n">
-        <v>35.877602</v>
+        <v>42.212399</v>
       </c>
       <c r="H295" t="n">
-        <v>-78.787498</v>
+        <v>-83.35340100000001</v>
       </c>
     </row>
     <row r="296">
       <c r="A296" s="1" t="inlineStr">
         <is>
-          <t>GDL</t>
+          <t>RDU</t>
         </is>
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>Guadalajara, Mexico</t>
+          <t>Durham, United States</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
@@ -11492,35 +11492,35 @@
       </c>
       <c r="D296" t="inlineStr">
         <is>
-          <t>Guadalajara</t>
+          <t>Raleigh/Durham</t>
         </is>
       </c>
       <c r="E296" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F296" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G296" t="n">
-        <v>20.521799</v>
+        <v>35.877602</v>
       </c>
       <c r="H296" t="n">
-        <v>-103.310997</v>
+        <v>-78.787498</v>
       </c>
     </row>
     <row r="297">
       <c r="A297" s="1" t="inlineStr">
         <is>
-          <t>YHZ</t>
+          <t>GDL</t>
         </is>
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>Halifax, Canada</t>
+          <t>Guadalajara, Mexico</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
@@ -11530,35 +11530,35 @@
       </c>
       <c r="D297" t="inlineStr">
         <is>
-          <t>Halifax</t>
+          <t>Guadalajara</t>
         </is>
       </c>
       <c r="E297" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F297" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>MX</t>
         </is>
       </c>
       <c r="G297" t="n">
-        <v>44.880798</v>
+        <v>20.521799</v>
       </c>
       <c r="H297" t="n">
-        <v>-63.508598</v>
+        <v>-103.310997</v>
       </c>
     </row>
     <row r="298">
       <c r="A298" s="1" t="inlineStr">
         <is>
-          <t>GUA</t>
+          <t>YHZ</t>
         </is>
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>Guatemala City, Guatemala</t>
+          <t>Halifax, Canada</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
@@ -11568,35 +11568,35 @@
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t>Guatemala City</t>
+          <t>Halifax</t>
         </is>
       </c>
       <c r="E298" t="inlineStr">
         <is>
-          <t>Guatemala</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F298" t="inlineStr">
         <is>
-          <t>GT</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="G298" t="n">
-        <v>14.5833</v>
+        <v>44.880798</v>
       </c>
       <c r="H298" t="n">
-        <v>-90.527496</v>
+        <v>-63.508598</v>
       </c>
     </row>
     <row r="299">
       <c r="A299" s="1" t="inlineStr">
         <is>
-          <t>HNL</t>
+          <t>GUA</t>
         </is>
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>Honolulu, United States</t>
+          <t>Guatemala City, Guatemala</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
@@ -11606,35 +11606,35 @@
       </c>
       <c r="D299" t="inlineStr">
         <is>
-          <t>Honolulu</t>
+          <t>Guatemala City</t>
         </is>
       </c>
       <c r="E299" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Guatemala</t>
         </is>
       </c>
       <c r="F299" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>GT</t>
         </is>
       </c>
       <c r="G299" t="n">
-        <v>21.318701</v>
+        <v>14.5833</v>
       </c>
       <c r="H299" t="n">
-        <v>-157.921997</v>
+        <v>-90.527496</v>
       </c>
     </row>
     <row r="300">
       <c r="A300" s="1" t="inlineStr">
         <is>
-          <t>IAH</t>
+          <t>HNL</t>
         </is>
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>Houston, United States</t>
+          <t>Honolulu, United States</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
@@ -11644,7 +11644,7 @@
       </c>
       <c r="D300" t="inlineStr">
         <is>
-          <t>Houston</t>
+          <t>Honolulu</t>
         </is>
       </c>
       <c r="E300" t="inlineStr">
@@ -11658,21 +11658,21 @@
         </is>
       </c>
       <c r="G300" t="n">
-        <v>29.9844</v>
+        <v>21.318701</v>
       </c>
       <c r="H300" t="n">
-        <v>-95.34139999999999</v>
+        <v>-157.921997</v>
       </c>
     </row>
     <row r="301">
       <c r="A301" s="1" t="inlineStr">
         <is>
-          <t>IND</t>
+          <t>IAH</t>
         </is>
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>Indianapolis, United States</t>
+          <t>Houston, United States</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
@@ -11682,7 +11682,7 @@
       </c>
       <c r="D301" t="inlineStr">
         <is>
-          <t>Indianapolis</t>
+          <t>Houston</t>
         </is>
       </c>
       <c r="E301" t="inlineStr">
@@ -11696,21 +11696,21 @@
         </is>
       </c>
       <c r="G301" t="n">
-        <v>39.7173</v>
+        <v>29.9844</v>
       </c>
       <c r="H301" t="n">
-        <v>-86.294403</v>
+        <v>-95.34139999999999</v>
       </c>
     </row>
     <row r="302">
       <c r="A302" s="1" t="inlineStr">
         <is>
-          <t>JAX</t>
+          <t>IND</t>
         </is>
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>Jacksonville, United States</t>
+          <t>Indianapolis, United States</t>
         </is>
       </c>
       <c r="C302" t="inlineStr">
@@ -11720,7 +11720,7 @@
       </c>
       <c r="D302" t="inlineStr">
         <is>
-          <t>Jacksonville</t>
+          <t>Indianapolis</t>
         </is>
       </c>
       <c r="E302" t="inlineStr">
@@ -11734,21 +11734,21 @@
         </is>
       </c>
       <c r="G302" t="n">
-        <v>30.494101</v>
+        <v>39.7173</v>
       </c>
       <c r="H302" t="n">
-        <v>-81.68789700000001</v>
+        <v>-86.294403</v>
       </c>
     </row>
     <row r="303">
       <c r="A303" s="1" t="inlineStr">
         <is>
-          <t>MCI</t>
+          <t>JAX</t>
         </is>
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>Kansas City, United States</t>
+          <t>Jacksonville, United States</t>
         </is>
       </c>
       <c r="C303" t="inlineStr">
@@ -11758,7 +11758,7 @@
       </c>
       <c r="D303" t="inlineStr">
         <is>
-          <t>Kansas City</t>
+          <t>Jacksonville</t>
         </is>
       </c>
       <c r="E303" t="inlineStr">
@@ -11772,21 +11772,21 @@
         </is>
       </c>
       <c r="G303" t="n">
-        <v>39.2976</v>
+        <v>30.494101</v>
       </c>
       <c r="H303" t="n">
-        <v>-94.713898</v>
+        <v>-81.68789700000001</v>
       </c>
     </row>
     <row r="304">
       <c r="A304" s="1" t="inlineStr">
         <is>
-          <t>KIN</t>
+          <t>MCI</t>
         </is>
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>Kingston, Jamaica</t>
+          <t>Kansas City, United States</t>
         </is>
       </c>
       <c r="C304" t="inlineStr">
@@ -11796,35 +11796,35 @@
       </c>
       <c r="D304" t="inlineStr">
         <is>
-          <t>Kingston</t>
+          <t>Kansas City</t>
         </is>
       </c>
       <c r="E304" t="inlineStr">
         <is>
-          <t>Jamaica</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F304" t="inlineStr">
         <is>
-          <t>JM</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G304" t="n">
-        <v>17.935699</v>
+        <v>39.2976</v>
       </c>
       <c r="H304" t="n">
-        <v>-76.787498</v>
+        <v>-94.713898</v>
       </c>
     </row>
     <row r="305">
       <c r="A305" s="1" t="inlineStr">
         <is>
-          <t>LAS</t>
+          <t>KIN</t>
         </is>
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>Las Vegas, United States</t>
+          <t>Kingston, Jamaica</t>
         </is>
       </c>
       <c r="C305" t="inlineStr">
@@ -11834,35 +11834,35 @@
       </c>
       <c r="D305" t="inlineStr">
         <is>
-          <t>Las Vegas</t>
+          <t>Kingston</t>
         </is>
       </c>
       <c r="E305" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Jamaica</t>
         </is>
       </c>
       <c r="F305" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>JM</t>
         </is>
       </c>
       <c r="G305" t="n">
-        <v>36.080101</v>
+        <v>17.935699</v>
       </c>
       <c r="H305" t="n">
-        <v>-115.152</v>
+        <v>-76.787498</v>
       </c>
     </row>
     <row r="306">
       <c r="A306" s="1" t="inlineStr">
         <is>
-          <t>LAX</t>
+          <t>LAS</t>
         </is>
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>Los Angeles, United States</t>
+          <t>Las Vegas, United States</t>
         </is>
       </c>
       <c r="C306" t="inlineStr">
@@ -11872,7 +11872,7 @@
       </c>
       <c r="D306" t="inlineStr">
         <is>
-          <t>Los Angeles</t>
+          <t>Las Vegas</t>
         </is>
       </c>
       <c r="E306" t="inlineStr">
@@ -11886,21 +11886,21 @@
         </is>
       </c>
       <c r="G306" t="n">
-        <v>33.942501</v>
+        <v>36.080101</v>
       </c>
       <c r="H306" t="n">
-        <v>-118.407997</v>
+        <v>-115.152</v>
       </c>
     </row>
     <row r="307">
       <c r="A307" s="1" t="inlineStr">
         <is>
-          <t>MEM</t>
+          <t>LAX</t>
         </is>
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>Memphis, United States</t>
+          <t>Los Angeles, United States</t>
         </is>
       </c>
       <c r="C307" t="inlineStr">
@@ -11910,7 +11910,7 @@
       </c>
       <c r="D307" t="inlineStr">
         <is>
-          <t>Memphis</t>
+          <t>Los Angeles</t>
         </is>
       </c>
       <c r="E307" t="inlineStr">
@@ -11924,21 +11924,21 @@
         </is>
       </c>
       <c r="G307" t="n">
-        <v>35.0424</v>
+        <v>33.942501</v>
       </c>
       <c r="H307" t="n">
-        <v>-89.97669999999999</v>
+        <v>-118.407997</v>
       </c>
     </row>
     <row r="308">
       <c r="A308" s="1" t="inlineStr">
         <is>
-          <t>MEX</t>
+          <t>MEM</t>
         </is>
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>Mexico City, Mexico</t>
+          <t>Memphis, United States</t>
         </is>
       </c>
       <c r="C308" t="inlineStr">
@@ -11948,35 +11948,35 @@
       </c>
       <c r="D308" t="inlineStr">
         <is>
-          <t>Mexico City</t>
+          <t>Memphis</t>
         </is>
       </c>
       <c r="E308" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F308" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G308" t="n">
-        <v>19.4363</v>
+        <v>35.0424</v>
       </c>
       <c r="H308" t="n">
-        <v>-99.072098</v>
+        <v>-89.97669999999999</v>
       </c>
     </row>
     <row r="309">
       <c r="A309" s="1" t="inlineStr">
         <is>
-          <t>MIA</t>
+          <t>MEX</t>
         </is>
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>Miami, United States</t>
+          <t>Mexico City, Mexico</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
@@ -11986,35 +11986,35 @@
       </c>
       <c r="D309" t="inlineStr">
         <is>
-          <t>Miami</t>
+          <t>Mexico City</t>
         </is>
       </c>
       <c r="E309" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F309" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>MX</t>
         </is>
       </c>
       <c r="G309" t="n">
-        <v>25.7932</v>
+        <v>19.4363</v>
       </c>
       <c r="H309" t="n">
-        <v>-80.290604</v>
+        <v>-99.072098</v>
       </c>
     </row>
     <row r="310">
       <c r="A310" s="1" t="inlineStr">
         <is>
-          <t>MSP</t>
+          <t>MIA</t>
         </is>
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>Minneapolis, United States</t>
+          <t>Miami, United States</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
@@ -12024,7 +12024,7 @@
       </c>
       <c r="D310" t="inlineStr">
         <is>
-          <t>Minneapolis</t>
+          <t>Miami</t>
         </is>
       </c>
       <c r="E310" t="inlineStr">
@@ -12038,21 +12038,21 @@
         </is>
       </c>
       <c r="G310" t="n">
-        <v>44.882</v>
+        <v>25.7932</v>
       </c>
       <c r="H310" t="n">
-        <v>-93.221802</v>
+        <v>-80.290604</v>
       </c>
     </row>
     <row r="311">
       <c r="A311" s="1" t="inlineStr">
         <is>
-          <t>YUL</t>
+          <t>MSP</t>
         </is>
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>Montréal, Canada</t>
+          <t>Minneapolis, United States</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
@@ -12062,35 +12062,35 @@
       </c>
       <c r="D311" t="inlineStr">
         <is>
-          <t>Montreal</t>
+          <t>Minneapolis</t>
         </is>
       </c>
       <c r="E311" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F311" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G311" t="n">
-        <v>45.4706</v>
+        <v>44.882</v>
       </c>
       <c r="H311" t="n">
-        <v>-73.740799</v>
+        <v>-93.221802</v>
       </c>
     </row>
     <row r="312">
       <c r="A312" s="1" t="inlineStr">
         <is>
-          <t>BNA</t>
+          <t>YUL</t>
         </is>
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>Nashville, United States</t>
+          <t>Montréal, Canada</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
@@ -12100,35 +12100,35 @@
       </c>
       <c r="D312" t="inlineStr">
         <is>
-          <t>Nashville</t>
+          <t>Montreal</t>
         </is>
       </c>
       <c r="E312" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F312" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="G312" t="n">
-        <v>36.1245</v>
+        <v>45.4706</v>
       </c>
       <c r="H312" t="n">
-        <v>-86.6782</v>
+        <v>-73.740799</v>
       </c>
     </row>
     <row r="313">
       <c r="A313" s="1" t="inlineStr">
         <is>
-          <t>EWR</t>
+          <t>BNA</t>
         </is>
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>Newark, United States</t>
+          <t>Nashville, United States</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
@@ -12138,7 +12138,7 @@
       </c>
       <c r="D313" t="inlineStr">
         <is>
-          <t>Newark</t>
+          <t>Nashville</t>
         </is>
       </c>
       <c r="E313" t="inlineStr">
@@ -12152,21 +12152,21 @@
         </is>
       </c>
       <c r="G313" t="n">
-        <v>40.692501</v>
+        <v>36.1245</v>
       </c>
       <c r="H313" t="n">
-        <v>-74.168701</v>
+        <v>-86.6782</v>
       </c>
     </row>
     <row r="314">
       <c r="A314" s="1" t="inlineStr">
         <is>
-          <t>ORF</t>
+          <t>EWR</t>
         </is>
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>Norfolk, United States</t>
+          <t>Newark, United States</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
@@ -12176,7 +12176,7 @@
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>Norfolk</t>
+          <t>Newark</t>
         </is>
       </c>
       <c r="E314" t="inlineStr">
@@ -12190,21 +12190,21 @@
         </is>
       </c>
       <c r="G314" t="n">
-        <v>36.8946</v>
+        <v>40.692501</v>
       </c>
       <c r="H314" t="n">
-        <v>-76.20120199999999</v>
+        <v>-74.168701</v>
       </c>
     </row>
     <row r="315">
       <c r="A315" s="1" t="inlineStr">
         <is>
-          <t>OKC</t>
+          <t>ORF</t>
         </is>
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>Oklahoma City, United States</t>
+          <t>Norfolk, United States</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
@@ -12214,7 +12214,7 @@
       </c>
       <c r="D315" t="inlineStr">
         <is>
-          <t>Oklahoma City</t>
+          <t>Norfolk</t>
         </is>
       </c>
       <c r="E315" t="inlineStr">
@@ -12228,21 +12228,21 @@
         </is>
       </c>
       <c r="G315" t="n">
-        <v>35.393101</v>
+        <v>36.8946</v>
       </c>
       <c r="H315" t="n">
-        <v>-97.6007</v>
+        <v>-76.20120199999999</v>
       </c>
     </row>
     <row r="316">
       <c r="A316" s="1" t="inlineStr">
         <is>
-          <t>OMA</t>
+          <t>OKC</t>
         </is>
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>Omaha, United States</t>
+          <t>Oklahoma City, United States</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
@@ -12252,7 +12252,7 @@
       </c>
       <c r="D316" t="inlineStr">
         <is>
-          <t>Omaha</t>
+          <t>Oklahoma City</t>
         </is>
       </c>
       <c r="E316" t="inlineStr">
@@ -12266,21 +12266,21 @@
         </is>
       </c>
       <c r="G316" t="n">
-        <v>41.3032</v>
+        <v>35.393101</v>
       </c>
       <c r="H316" t="n">
-        <v>-95.894096</v>
+        <v>-97.6007</v>
       </c>
     </row>
     <row r="317">
       <c r="A317" s="1" t="inlineStr">
         <is>
-          <t>PHL</t>
+          <t>OMA</t>
         </is>
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>Philadelphia, United States</t>
+          <t>Omaha, United States</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
@@ -12290,7 +12290,7 @@
       </c>
       <c r="D317" t="inlineStr">
         <is>
-          <t>Philadelphia</t>
+          <t>Omaha</t>
         </is>
       </c>
       <c r="E317" t="inlineStr">
@@ -12304,21 +12304,21 @@
         </is>
       </c>
       <c r="G317" t="n">
-        <v>39.871899</v>
+        <v>41.3032</v>
       </c>
       <c r="H317" t="n">
-        <v>-75.241096</v>
+        <v>-95.894096</v>
       </c>
     </row>
     <row r="318">
       <c r="A318" s="1" t="inlineStr">
         <is>
-          <t>PHX</t>
+          <t>PHL</t>
         </is>
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>Phoenix, United States</t>
+          <t>Philadelphia, United States</t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
@@ -12328,7 +12328,7 @@
       </c>
       <c r="D318" t="inlineStr">
         <is>
-          <t>Phoenix</t>
+          <t>Philadelphia</t>
         </is>
       </c>
       <c r="E318" t="inlineStr">
@@ -12342,21 +12342,21 @@
         </is>
       </c>
       <c r="G318" t="n">
-        <v>33.434299</v>
+        <v>39.871899</v>
       </c>
       <c r="H318" t="n">
-        <v>-112.012001</v>
+        <v>-75.241096</v>
       </c>
     </row>
     <row r="319">
       <c r="A319" s="1" t="inlineStr">
         <is>
-          <t>SDQ</t>
+          <t>PHX</t>
         </is>
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>Santo Domingo, Dominican Republic</t>
+          <t>Phoenix, United States</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
@@ -12366,35 +12366,35 @@
       </c>
       <c r="D319" t="inlineStr">
         <is>
-          <t>Santo Domingo</t>
+          <t>Phoenix</t>
         </is>
       </c>
       <c r="E319" t="inlineStr">
         <is>
-          <t>Dominican Republic</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F319" t="inlineStr">
         <is>
-          <t>DO</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G319" t="n">
-        <v>18.429701</v>
+        <v>33.434299</v>
       </c>
       <c r="H319" t="n">
-        <v>-69.66889999999999</v>
+        <v>-112.012001</v>
       </c>
     </row>
     <row r="320">
       <c r="A320" s="1" t="inlineStr">
         <is>
-          <t>PIT</t>
+          <t>SDQ</t>
         </is>
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>Pittsburgh, United States</t>
+          <t>Santo Domingo, Dominican Republic</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
@@ -12404,35 +12404,35 @@
       </c>
       <c r="D320" t="inlineStr">
         <is>
-          <t>Pittsburgh</t>
+          <t>Santo Domingo</t>
         </is>
       </c>
       <c r="E320" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Dominican Republic</t>
         </is>
       </c>
       <c r="F320" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>DO</t>
         </is>
       </c>
       <c r="G320" t="n">
-        <v>40.491501</v>
+        <v>18.429701</v>
       </c>
       <c r="H320" t="n">
-        <v>-80.23290299999999</v>
+        <v>-69.66889999999999</v>
       </c>
     </row>
     <row r="321">
       <c r="A321" s="1" t="inlineStr">
         <is>
-          <t>PDX</t>
+          <t>PIT</t>
         </is>
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>Portland, United States</t>
+          <t>Pittsburgh, United States</t>
         </is>
       </c>
       <c r="C321" t="inlineStr">
@@ -12442,7 +12442,7 @@
       </c>
       <c r="D321" t="inlineStr">
         <is>
-          <t>Portland</t>
+          <t>Pittsburgh</t>
         </is>
       </c>
       <c r="E321" t="inlineStr">
@@ -12456,21 +12456,21 @@
         </is>
       </c>
       <c r="G321" t="n">
-        <v>45.588699</v>
+        <v>40.491501</v>
       </c>
       <c r="H321" t="n">
-        <v>-122.598</v>
+        <v>-80.23290299999999</v>
       </c>
     </row>
     <row r="322">
       <c r="A322" s="1" t="inlineStr">
         <is>
-          <t>QRO</t>
+          <t>PDX</t>
         </is>
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>Queretaro, Mexico</t>
+          <t>Portland, United States</t>
         </is>
       </c>
       <c r="C322" t="inlineStr">
@@ -12480,35 +12480,35 @@
       </c>
       <c r="D322" t="inlineStr">
         <is>
-          <t>Queretaro</t>
+          <t>Portland</t>
         </is>
       </c>
       <c r="E322" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F322" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G322" t="n">
-        <v>20.6173</v>
+        <v>45.588699</v>
       </c>
       <c r="H322" t="n">
-        <v>-100.185997</v>
+        <v>-122.598</v>
       </c>
     </row>
     <row r="323">
       <c r="A323" s="1" t="inlineStr">
         <is>
-          <t>RIC</t>
+          <t>QRO</t>
         </is>
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>Richmond, United States</t>
+          <t>Queretaro, Mexico</t>
         </is>
       </c>
       <c r="C323" t="inlineStr">
@@ -12518,35 +12518,35 @@
       </c>
       <c r="D323" t="inlineStr">
         <is>
-          <t>Richmond</t>
+          <t>Queretaro</t>
         </is>
       </c>
       <c r="E323" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F323" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>MX</t>
         </is>
       </c>
       <c r="G323" t="n">
-        <v>37.505199</v>
+        <v>20.6173</v>
       </c>
       <c r="H323" t="n">
-        <v>-77.31970200000001</v>
+        <v>-100.185997</v>
       </c>
     </row>
     <row r="324">
       <c r="A324" s="1" t="inlineStr">
         <is>
-          <t>SMF</t>
+          <t>RIC</t>
         </is>
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>Sacramento, United States</t>
+          <t>Richmond, United States</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
@@ -12556,7 +12556,7 @@
       </c>
       <c r="D324" t="inlineStr">
         <is>
-          <t>Sacramento</t>
+          <t>Richmond</t>
         </is>
       </c>
       <c r="E324" t="inlineStr">
@@ -12570,21 +12570,21 @@
         </is>
       </c>
       <c r="G324" t="n">
-        <v>38.6954</v>
+        <v>37.505199</v>
       </c>
       <c r="H324" t="n">
-        <v>-121.591003</v>
+        <v>-77.31970200000001</v>
       </c>
     </row>
     <row r="325">
       <c r="A325" s="1" t="inlineStr">
         <is>
-          <t>SLC</t>
+          <t>SMF</t>
         </is>
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>Salt Lake City, United States</t>
+          <t>Sacramento, United States</t>
         </is>
       </c>
       <c r="C325" t="inlineStr">
@@ -12594,7 +12594,7 @@
       </c>
       <c r="D325" t="inlineStr">
         <is>
-          <t>Salt Lake City</t>
+          <t>Sacramento</t>
         </is>
       </c>
       <c r="E325" t="inlineStr">
@@ -12608,21 +12608,21 @@
         </is>
       </c>
       <c r="G325" t="n">
-        <v>40.788399</v>
+        <v>38.6954</v>
       </c>
       <c r="H325" t="n">
-        <v>-111.977997</v>
+        <v>-121.591003</v>
       </c>
     </row>
     <row r="326">
       <c r="A326" s="1" t="inlineStr">
         <is>
-          <t>SAT</t>
+          <t>SLC</t>
         </is>
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>San Antonio, United States</t>
+          <t>Salt Lake City, United States</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
@@ -12632,7 +12632,7 @@
       </c>
       <c r="D326" t="inlineStr">
         <is>
-          <t>San Antonio</t>
+          <t>Salt Lake City</t>
         </is>
       </c>
       <c r="E326" t="inlineStr">
@@ -12646,21 +12646,21 @@
         </is>
       </c>
       <c r="G326" t="n">
-        <v>29.533701</v>
+        <v>40.788399</v>
       </c>
       <c r="H326" t="n">
-        <v>-98.469803</v>
+        <v>-111.977997</v>
       </c>
     </row>
     <row r="327">
       <c r="A327" s="1" t="inlineStr">
         <is>
-          <t>SAN</t>
+          <t>SAT</t>
         </is>
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>San Diego, United States</t>
+          <t>San Antonio, United States</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
@@ -12670,7 +12670,7 @@
       </c>
       <c r="D327" t="inlineStr">
         <is>
-          <t>San Diego</t>
+          <t>San Antonio</t>
         </is>
       </c>
       <c r="E327" t="inlineStr">
@@ -12684,21 +12684,21 @@
         </is>
       </c>
       <c r="G327" t="n">
-        <v>32.733601</v>
+        <v>29.533701</v>
       </c>
       <c r="H327" t="n">
-        <v>-117.190002</v>
+        <v>-98.469803</v>
       </c>
     </row>
     <row r="328">
       <c r="A328" s="1" t="inlineStr">
         <is>
-          <t>SFO</t>
+          <t>SAN</t>
         </is>
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>San Francisco, United States</t>
+          <t>San Diego, United States</t>
         </is>
       </c>
       <c r="C328" t="inlineStr">
@@ -12708,7 +12708,7 @@
       </c>
       <c r="D328" t="inlineStr">
         <is>
-          <t>San Francisco</t>
+          <t>San Diego</t>
         </is>
       </c>
       <c r="E328" t="inlineStr">
@@ -12722,21 +12722,21 @@
         </is>
       </c>
       <c r="G328" t="n">
-        <v>37.618999</v>
+        <v>32.733601</v>
       </c>
       <c r="H328" t="n">
-        <v>-122.375</v>
+        <v>-117.190002</v>
       </c>
     </row>
     <row r="329">
       <c r="A329" s="1" t="inlineStr">
         <is>
-          <t>SJC</t>
+          <t>SFO</t>
         </is>
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>San Jose, United States</t>
+          <t>San Francisco, United States</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
@@ -12746,7 +12746,7 @@
       </c>
       <c r="D329" t="inlineStr">
         <is>
-          <t>San Jose</t>
+          <t>San Francisco</t>
         </is>
       </c>
       <c r="E329" t="inlineStr">
@@ -12760,21 +12760,21 @@
         </is>
       </c>
       <c r="G329" t="n">
-        <v>37.362598</v>
+        <v>37.618999</v>
       </c>
       <c r="H329" t="n">
-        <v>-121.929001</v>
+        <v>-122.375</v>
       </c>
     </row>
     <row r="330">
       <c r="A330" s="1" t="inlineStr">
         <is>
-          <t>YXE</t>
+          <t>SJC</t>
         </is>
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>Saskatoon, Canada</t>
+          <t>San Jose, United States</t>
         </is>
       </c>
       <c r="C330" t="inlineStr">
@@ -12784,35 +12784,35 @@
       </c>
       <c r="D330" t="inlineStr">
         <is>
-          <t>Saskatoon</t>
+          <t>San Jose</t>
         </is>
       </c>
       <c r="E330" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F330" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G330" t="n">
-        <v>52.170799</v>
+        <v>37.362598</v>
       </c>
       <c r="H330" t="n">
-        <v>-106.699997</v>
+        <v>-121.929001</v>
       </c>
     </row>
     <row r="331">
       <c r="A331" s="1" t="inlineStr">
         <is>
-          <t>SEA</t>
+          <t>YXE</t>
         </is>
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>Seattle, United States</t>
+          <t>Saskatoon, Canada</t>
         </is>
       </c>
       <c r="C331" t="inlineStr">
@@ -12822,35 +12822,35 @@
       </c>
       <c r="D331" t="inlineStr">
         <is>
-          <t>Seattle</t>
+          <t>Saskatoon</t>
         </is>
       </c>
       <c r="E331" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F331" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="G331" t="n">
-        <v>47.449001</v>
+        <v>52.170799</v>
       </c>
       <c r="H331" t="n">
-        <v>-122.308998</v>
+        <v>-106.699997</v>
       </c>
     </row>
     <row r="332">
       <c r="A332" s="1" t="inlineStr">
         <is>
-          <t>FSD</t>
+          <t>SEA</t>
         </is>
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>Sioux Falls, United States</t>
+          <t>Seattle, United States</t>
         </is>
       </c>
       <c r="C332" t="inlineStr">
@@ -12860,7 +12860,7 @@
       </c>
       <c r="D332" t="inlineStr">
         <is>
-          <t>Sioux Falls</t>
+          <t>Seattle</t>
         </is>
       </c>
       <c r="E332" t="inlineStr">
@@ -12874,21 +12874,21 @@
         </is>
       </c>
       <c r="G332" t="n">
-        <v>43.582001</v>
+        <v>47.449001</v>
       </c>
       <c r="H332" t="n">
-        <v>-96.74189800000001</v>
+        <v>-122.308998</v>
       </c>
     </row>
     <row r="333">
       <c r="A333" s="1" t="inlineStr">
         <is>
-          <t>BGI</t>
+          <t>FSD</t>
         </is>
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>Bridgetown, Barbados</t>
+          <t>Sioux Falls, United States</t>
         </is>
       </c>
       <c r="C333" t="inlineStr">
@@ -12898,35 +12898,35 @@
       </c>
       <c r="D333" t="inlineStr">
         <is>
-          <t>Bridgetown</t>
+          <t>Sioux Falls</t>
         </is>
       </c>
       <c r="E333" t="inlineStr">
         <is>
-          <t>Barbados</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F333" t="inlineStr">
         <is>
-          <t>BB</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G333" t="n">
-        <v>13.0746</v>
+        <v>43.582001</v>
       </c>
       <c r="H333" t="n">
-        <v>-59.4925</v>
+        <v>-96.74189800000001</v>
       </c>
     </row>
     <row r="334">
       <c r="A334" s="1" t="inlineStr">
         <is>
-          <t>STL</t>
+          <t>BGI</t>
         </is>
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>St. Louis, United States</t>
+          <t>Bridgetown, Barbados</t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
@@ -12936,35 +12936,35 @@
       </c>
       <c r="D334" t="inlineStr">
         <is>
-          <t>St Louis</t>
+          <t>Bridgetown</t>
         </is>
       </c>
       <c r="E334" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Barbados</t>
         </is>
       </c>
       <c r="F334" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>BB</t>
         </is>
       </c>
       <c r="G334" t="n">
-        <v>38.748699</v>
+        <v>13.0746</v>
       </c>
       <c r="H334" t="n">
-        <v>-90.370003</v>
+        <v>-59.4925</v>
       </c>
     </row>
     <row r="335">
       <c r="A335" s="1" t="inlineStr">
         <is>
-          <t>TLH</t>
+          <t>STL</t>
         </is>
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>Tallahassee, United States</t>
+          <t>St. Louis, United States</t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
@@ -12974,7 +12974,7 @@
       </c>
       <c r="D335" t="inlineStr">
         <is>
-          <t>Tallahassee</t>
+          <t>St Louis</t>
         </is>
       </c>
       <c r="E335" t="inlineStr">
@@ -12988,21 +12988,21 @@
         </is>
       </c>
       <c r="G335" t="n">
-        <v>30.3965</v>
+        <v>38.748699</v>
       </c>
       <c r="H335" t="n">
-        <v>-84.35030399999999</v>
+        <v>-90.370003</v>
       </c>
     </row>
     <row r="336">
       <c r="A336" s="1" t="inlineStr">
         <is>
-          <t>STI</t>
+          <t>TLH</t>
         </is>
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>Santiago de los Caballeros, Dominican Republic</t>
+          <t>Tallahassee, United States</t>
         </is>
       </c>
       <c r="C336" t="inlineStr">
@@ -13012,35 +13012,35 @@
       </c>
       <c r="D336" t="inlineStr">
         <is>
-          <t>Santiago</t>
+          <t>Tallahassee</t>
         </is>
       </c>
       <c r="E336" t="inlineStr">
         <is>
-          <t>Dominican Republic</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F336" t="inlineStr">
         <is>
-          <t>DO</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G336" t="n">
-        <v>19.406099</v>
+        <v>30.3965</v>
       </c>
       <c r="H336" t="n">
-        <v>-70.604698</v>
+        <v>-84.35030399999999</v>
       </c>
     </row>
     <row r="337">
       <c r="A337" s="1" t="inlineStr">
         <is>
-          <t>TPA</t>
+          <t>STI</t>
         </is>
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>Tampa, United States</t>
+          <t>Santiago de los Caballeros, Dominican Republic</t>
         </is>
       </c>
       <c r="C337" t="inlineStr">
@@ -13050,35 +13050,35 @@
       </c>
       <c r="D337" t="inlineStr">
         <is>
-          <t>Tampa</t>
+          <t>Santiago</t>
         </is>
       </c>
       <c r="E337" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Dominican Republic</t>
         </is>
       </c>
       <c r="F337" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>DO</t>
         </is>
       </c>
       <c r="G337" t="n">
-        <v>27.9755</v>
+        <v>19.406099</v>
       </c>
       <c r="H337" t="n">
-        <v>-82.533203</v>
+        <v>-70.604698</v>
       </c>
     </row>
     <row r="338">
       <c r="A338" s="1" t="inlineStr">
         <is>
-          <t>YYZ</t>
+          <t>TPA</t>
         </is>
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t>Toronto, Canada</t>
+          <t>Tampa, United States</t>
         </is>
       </c>
       <c r="C338" t="inlineStr">
@@ -13088,35 +13088,35 @@
       </c>
       <c r="D338" t="inlineStr">
         <is>
-          <t>Toronto</t>
+          <t>Tampa</t>
         </is>
       </c>
       <c r="E338" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F338" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G338" t="n">
-        <v>43.6772</v>
+        <v>27.9755</v>
       </c>
       <c r="H338" t="n">
-        <v>-79.6306</v>
+        <v>-82.533203</v>
       </c>
     </row>
     <row r="339">
       <c r="A339" s="1" t="inlineStr">
         <is>
-          <t>YVR</t>
+          <t>YYZ</t>
         </is>
       </c>
       <c r="B339" t="inlineStr">
         <is>
-          <t>Vancouver, Canada</t>
+          <t>Toronto, Canada</t>
         </is>
       </c>
       <c r="C339" t="inlineStr">
@@ -13126,7 +13126,7 @@
       </c>
       <c r="D339" t="inlineStr">
         <is>
-          <t>Vancouver</t>
+          <t>Toronto</t>
         </is>
       </c>
       <c r="E339" t="inlineStr">
@@ -13140,21 +13140,21 @@
         </is>
       </c>
       <c r="G339" t="n">
-        <v>49.193901</v>
+        <v>43.6772</v>
       </c>
       <c r="H339" t="n">
-        <v>-123.183998</v>
+        <v>-79.6306</v>
       </c>
     </row>
     <row r="340">
       <c r="A340" s="1" t="inlineStr">
         <is>
-          <t>SJU</t>
+          <t>YVR</t>
         </is>
       </c>
       <c r="B340" t="inlineStr">
         <is>
-          <t>San Juan, Puerto Rico</t>
+          <t>Vancouver, Canada</t>
         </is>
       </c>
       <c r="C340" t="inlineStr">
@@ -13164,35 +13164,35 @@
       </c>
       <c r="D340" t="inlineStr">
         <is>
-          <t>San Juan</t>
+          <t>Vancouver</t>
         </is>
       </c>
       <c r="E340" t="inlineStr">
         <is>
-          <t>Puerto Rico</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F340" t="inlineStr">
         <is>
-          <t>PR</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="G340" t="n">
-        <v>18.4394</v>
+        <v>49.193901</v>
       </c>
       <c r="H340" t="n">
-        <v>-66.001801</v>
+        <v>-123.183998</v>
       </c>
     </row>
     <row r="341">
       <c r="A341" s="1" t="inlineStr">
         <is>
-          <t>YWG</t>
+          <t>SJU</t>
         </is>
       </c>
       <c r="B341" t="inlineStr">
         <is>
-          <t>Winnipeg, Canada</t>
+          <t>San Juan, Puerto Rico</t>
         </is>
       </c>
       <c r="C341" t="inlineStr">
@@ -13202,61 +13202,99 @@
       </c>
       <c r="D341" t="inlineStr">
         <is>
-          <t>Winnipeg</t>
+          <t>San Juan</t>
         </is>
       </c>
       <c r="E341" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>Puerto Rico</t>
         </is>
       </c>
       <c r="F341" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>PR</t>
         </is>
       </c>
       <c r="G341" t="n">
-        <v>49.91</v>
+        <v>18.4394</v>
       </c>
       <c r="H341" t="n">
-        <v>-97.23989899999999</v>
+        <v>-66.001801</v>
       </c>
     </row>
     <row r="342">
       <c r="A342" s="1" t="inlineStr">
         <is>
+          <t>YWG</t>
+        </is>
+      </c>
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>Winnipeg, Canada</t>
+        </is>
+      </c>
+      <c r="C342" t="inlineStr">
+        <is>
+          <t>North America</t>
+        </is>
+      </c>
+      <c r="D342" t="inlineStr">
+        <is>
+          <t>Winnipeg</t>
+        </is>
+      </c>
+      <c r="E342" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="F342" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="G342" t="n">
+        <v>49.91</v>
+      </c>
+      <c r="H342" t="n">
+        <v>-97.23989899999999</v>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" s="1" t="inlineStr">
+        <is>
           <t>CVG</t>
         </is>
       </c>
-      <c r="B342" t="inlineStr">
+      <c r="B343" t="inlineStr">
         <is>
           <t>Cincinnati, United States</t>
         </is>
       </c>
-      <c r="C342" t="inlineStr">
+      <c r="C343" t="inlineStr">
         <is>
           <t>North America</t>
         </is>
       </c>
-      <c r="D342" t="inlineStr">
+      <c r="D343" t="inlineStr">
         <is>
           <t>Hebron</t>
         </is>
       </c>
-      <c r="E342" t="inlineStr">
+      <c r="E343" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="F342" t="inlineStr">
+      <c r="F343" t="inlineStr">
         <is>
           <t>US</t>
         </is>
       </c>
-      <c r="G342" t="n">
+      <c r="G343" t="n">
         <v>39.048801</v>
       </c>
-      <c r="H342" t="n">
+      <c r="H343" t="n">
         <v>-84.667801</v>
       </c>
     </row>

</xml_diff>